<commit_message>
Final UI changes (settings,activity logs)
</commit_message>
<xml_diff>
--- a/backend/storage/output/excel/train-no/Rail_Madad_Report_3_Top_20_Trains_14-07-2026.xlsx
+++ b/backend/storage/output/excel/train-no/Rail_Madad_Report_3_Top_20_Trains_14-07-2026.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,27 +482,27 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>22503</t>
+          <t>19484</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>VIVEK EXPRESS [SUPERFAST]</t>
+          <t>SHC - ADI EXPRESS [MAIL EXPRESS]</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Northeast Frontier Railway</t>
+          <t>Western Railway</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>TINSUKIA DIVISION</t>
+          <t>AHMEDABAD DIVISION</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>51</t>
         </is>
       </c>
     </row>
@@ -514,27 +514,603 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>14115</t>
+          <t>15657</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>DADN-PRYJ EXP. [MAIL EXPRESS]</t>
+          <t>BRAHMAPUTRA MAIL [MAIL EXPRESS]</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>Northeast Frontier Railway</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>LUMDING DIVISION</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>22504</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>VIVEK EXPRESS [SUPERFAST]</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Northeast Frontier Railway</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>TINSUKIA DIVISION</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>15910</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>AVADH ASSAM EXPRESS [MAIL EXPRESS]</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Northeast Frontier Railway</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>TINSUKIA DIVISION</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>18478</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>YNRK-PURI EXPRESS [MAIL EXPRESS]</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>East Coast Railway</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>KHURDA DIVISION</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>04013</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>LKQ-ANVT SPL [TRAIN ON DEMAND]</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Northern Railway</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>DELHI DIVISION</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>12920</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>MALWA EXPRESS [SUPERFAST]</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Western Railway</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>RATLAM DIVISION</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>15909</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>AVADH ASSAM EXPRESS [MAIL EXPRESS]</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Northeast Frontier Railway</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>TINSUKIA DIVISION</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>22503</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>VIVEK EXPRESS [SUPERFAST]</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Northeast Frontier Railway</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>TINSUKIA DIVISION</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>03253</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>PNBE- CHZ EXPRESS SPL [TRAIN ON DEMAND]</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>East Central Railway</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>DANAPUR DIVISION</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>04313</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>MFP-YNRK SPL [TRAIN ON DEMAND]</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Northern Railway</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>MORADABAD DIVISION</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>12506</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>NORTHEAST EXPRESS [SUPERFAST]</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Northeast Frontier Railway</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>LUMDING DIVISION</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>12521</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>BJU-ERS RAPTI SAGAR EXP [SUPERFAST]</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>East Central Railway</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>SONEPUR DIVISION</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>19270</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>MFP - PBR EXP [MAIL EXPRESS]</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Western Railway</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>BHAVNAGAR DIVISION</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>01028</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>GKP-DR SPL [TRAIN ON DEMAND]</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Central Railway</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>BOMBAY DIVISION</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>12802</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>ANVT-PURI PURSHOTTAM [SUPERFAST]</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>East Coast Railway</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>KHURDA DIVISION</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>14116</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>PRYJ-DADN EXP. [MAIL EXPRESS]</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
           <t>North Central Railway</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>PRAYAGRAJ DIVISION</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>37</t>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>15023</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>GKP-YPR-EXP [MAIL EXPRESS]</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>North Eastern Railway</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>LUCKNOW DIVISION</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>03311</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>DHN -CDG SPECIAL [TRAIN ON DEMAND]</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>East Central Railway</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>DHANBAD DIVISION</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>12510</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>GHY-SMVB S/F EXPRESS [SUPERFAST]</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Northeast Frontier Railway</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>LUMDING DIVISION</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>23</t>
         </is>
       </c>
     </row>

</xml_diff>